<commit_message>
add new scenario data
</commit_message>
<xml_diff>
--- a/inventories/lci-sweet_sure.xlsx
+++ b/inventories/lci-sweet_sure.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10811"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10817"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/romain/GitHub/sweet_sure-2050-switzerland/inventories/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF103860-90D3-974C-B82B-3D59D2C1C84F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9634B431-0EB6-D549-BDA6-71D2490A93EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="42740" yWindow="-580" windowWidth="25800" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="lci" sheetId="6" r:id="rId1"/>
@@ -1259,9 +1259,6 @@
     <t>charger, electric passenger car</t>
   </si>
   <si>
-    <t>diesel, low-sulfur, import from Europe</t>
-  </si>
-  <si>
     <t>Combustion engine power: 287 [kW]. Power share from combustion engine: 100 [%]. Km over lifetime: 700000 [km]. Yearly mileage: 50000 [km/year]. Daily distance driven: 511 [km]. Daily operating time: 9 [hours]. Tank-to-wheel efficiency: 24 [%]. Tank-to-wheel energy consumption: 9105 [kj/km]. Fuel tank capacity: 1292 [kWh]. Maximum passenger capacity: 55 [unit]. Number of passengers onboard: 21 [unit]. Curb mass (excl. driver and cargo): 13074 [kg]. Driving mass (incl. driver and cargo): 15006 [kg].</t>
   </si>
   <si>
@@ -1578,6 +1575,9 @@
   </si>
   <si>
     <t xml:space="preserve">Electric motor power: 486 [kW]. Km over lifetime: 1000000 [km]. Yearly mileage: 60000 [km/year]. Autonomy on a full tank/battery: 150 [km]. Tank-to-wheel efficiency: 72 [%]. Tank-to-wheel energy consumption: 5447 [kj/km]. Battery capacity: 283 [kWh]. Mass of battery: 2364 [kg]. Available payload: 23696 [kg]. Payload: 8755 [kg]. Load factor: 36 [%]. Curb mass (excl. driver and cargo): 16228 [kg]. Driving mass (incl. driver and cargo): 25058 [kg]. </t>
+  </si>
+  <si>
+    <t>diesel, low-sulfur, import from Europe without Switzerland</t>
   </si>
 </sst>
 </file>
@@ -2710,7 +2710,7 @@
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="B39" s="3">
         <v>1.623727351164797E-7</v>
@@ -2726,7 +2726,7 @@
       </c>
       <c r="G39" s="2"/>
       <c r="H39" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
@@ -2810,7 +2810,7 @@
       </c>
       <c r="G43" s="2"/>
       <c r="H43" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">
@@ -3221,7 +3221,7 @@
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="B64" s="3">
         <v>6.8457290767903355E-12</v>
@@ -5254,7 +5254,7 @@
     </row>
     <row r="171" spans="1:10" s="50" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A171" s="50" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="B171" s="51">
         <f>6.1/43.4</f>
@@ -5264,13 +5264,13 @@
         <v>7</v>
       </c>
       <c r="E171" s="50" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="F171" s="50" t="s">
         <v>27</v>
       </c>
       <c r="G171" s="50" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="J171" s="51"/>
     </row>
@@ -5512,7 +5512,7 @@
     </row>
     <row r="190" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A190" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="B190" s="3">
         <v>5.8454184641932699E-7</v>
@@ -5528,7 +5528,7 @@
       </c>
       <c r="G190" s="2"/>
       <c r="H190" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
     </row>
     <row r="191" spans="1:8" x14ac:dyDescent="0.2">
@@ -5612,7 +5612,7 @@
       </c>
       <c r="G194" s="2"/>
       <c r="H194" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
     </row>
     <row r="195" spans="1:8" x14ac:dyDescent="0.2">
@@ -6023,7 +6023,7 @@
     </row>
     <row r="215" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A215" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="B215" s="3">
         <v>2.464462467644521E-11</v>
@@ -8056,7 +8056,7 @@
     </row>
     <row r="322" spans="1:8" s="50" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A322" s="50" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="B322" s="51">
         <f>9.3/43.4</f>
@@ -8066,13 +8066,13 @@
         <v>7</v>
       </c>
       <c r="E322" s="50" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="F322" s="50" t="s">
         <v>27</v>
       </c>
       <c r="G322" s="50" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
     </row>
     <row r="324" spans="1:8" s="50" customFormat="1" ht="16" x14ac:dyDescent="0.2">
@@ -8304,7 +8304,7 @@
     </row>
     <row r="340" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A340" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="B340" s="3">
         <v>6.4299603106125978E-7</v>
@@ -8320,7 +8320,7 @@
       </c>
       <c r="G340" s="2"/>
       <c r="H340" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
     </row>
     <row r="341" spans="1:8" x14ac:dyDescent="0.2">
@@ -8404,7 +8404,7 @@
       </c>
       <c r="G344" s="2"/>
       <c r="H344" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
     </row>
     <row r="345" spans="1:8" x14ac:dyDescent="0.2">
@@ -8815,7 +8815,7 @@
     </row>
     <row r="365" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A365" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="B365" s="3">
         <v>2.7109087144089735E-11</v>
@@ -10871,7 +10871,7 @@
     </row>
     <row r="473" spans="1:8" s="50" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A473" s="50" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="B473" s="51">
         <f>(9.3/43.4)*1.1</f>
@@ -10881,13 +10881,13 @@
         <v>7</v>
       </c>
       <c r="E473" s="50" t="s">
+        <v>485</v>
+      </c>
+      <c r="F473" s="50" t="s">
+        <v>27</v>
+      </c>
+      <c r="G473" s="50" t="s">
         <v>486</v>
-      </c>
-      <c r="F473" s="50" t="s">
-        <v>27</v>
-      </c>
-      <c r="G473" s="50" t="s">
-        <v>487</v>
       </c>
     </row>
     <row r="474" spans="1:8" s="50" customFormat="1" x14ac:dyDescent="0.2"/>
@@ -11120,7 +11120,7 @@
     </row>
     <row r="491" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A491" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="B491" s="3">
         <v>1.7861000862812767E-7</v>
@@ -11136,7 +11136,7 @@
       </c>
       <c r="G491" s="3"/>
       <c r="H491" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
     </row>
     <row r="492" spans="1:8" x14ac:dyDescent="0.2">
@@ -11220,7 +11220,7 @@
       </c>
       <c r="G495" s="3"/>
       <c r="H495" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
     </row>
     <row r="496" spans="1:8" x14ac:dyDescent="0.2">
@@ -11631,7 +11631,7 @@
     </row>
     <row r="516" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A516" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="B516" s="3">
         <v>7.5303019844693692E-12</v>
@@ -13682,12 +13682,12 @@
         <v>27</v>
       </c>
       <c r="G623" s="50" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
     </row>
     <row r="624" spans="1:8" s="50" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A624" s="50" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="B624" s="51">
         <f>6.1/43.4*1.1</f>
@@ -13697,13 +13697,13 @@
         <v>7</v>
       </c>
       <c r="E624" s="50" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="F624" s="50" t="s">
         <v>27</v>
       </c>
       <c r="G624" s="50" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
     </row>
     <row r="625" spans="1:8" s="50" customFormat="1" x14ac:dyDescent="0.2"/>
@@ -13966,7 +13966,7 @@
     </row>
     <row r="644" spans="1:8" s="50" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A644" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="B644" s="51">
         <v>4.796993006993007E-7</v>
@@ -13982,7 +13982,7 @@
       </c>
       <c r="G644" s="51"/>
       <c r="H644" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
     </row>
     <row r="645" spans="1:8" s="50" customFormat="1" x14ac:dyDescent="0.2">
@@ -14066,7 +14066,7 @@
       </c>
       <c r="G648" s="51"/>
       <c r="H648" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
     </row>
     <row r="649" spans="1:8" s="50" customFormat="1" x14ac:dyDescent="0.2">
@@ -14434,7 +14434,7 @@
     </row>
     <row r="667" spans="1:8" s="50" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A667" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="B667" s="51">
         <v>1.5376223776223777E-10</v>
@@ -16780,7 +16780,7 @@
     </row>
     <row r="802" spans="1:8" s="50" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A802" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="B802" s="51">
         <v>1.7269174825174825E-6</v>
@@ -16796,7 +16796,7 @@
       </c>
       <c r="G802" s="51"/>
       <c r="H802" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
     </row>
     <row r="803" spans="1:8" s="50" customFormat="1" x14ac:dyDescent="0.2">
@@ -16880,7 +16880,7 @@
       </c>
       <c r="G806" s="51"/>
       <c r="H806" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
     </row>
     <row r="807" spans="1:8" s="50" customFormat="1" x14ac:dyDescent="0.2">
@@ -17248,7 +17248,7 @@
     </row>
     <row r="825" spans="1:8" s="50" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A825" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="B825" s="51">
         <v>5.5354405594405596E-10</v>
@@ -19606,7 +19606,7 @@
     </row>
     <row r="960" spans="1:8" s="50" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A960" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="B960" s="51">
         <v>1.8996092307692309E-6</v>
@@ -19622,7 +19622,7 @@
       </c>
       <c r="G960" s="51"/>
       <c r="H960" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
     </row>
     <row r="961" spans="1:8" s="50" customFormat="1" x14ac:dyDescent="0.2">
@@ -19706,7 +19706,7 @@
       </c>
       <c r="G964" s="51"/>
       <c r="H964" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
     </row>
     <row r="965" spans="1:8" s="50" customFormat="1" x14ac:dyDescent="0.2">
@@ -20074,7 +20074,7 @@
     </row>
     <row r="983" spans="1:8" s="50" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A983" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="B983" s="51">
         <v>6.0889846153846164E-10</v>
@@ -22431,7 +22431,7 @@
     </row>
     <row r="1118" spans="1:8" s="50" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1118" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="B1118" s="51">
         <v>5.2766923076923077E-7</v>
@@ -22447,7 +22447,7 @@
       </c>
       <c r="G1118" s="51"/>
       <c r="H1118" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
     </row>
     <row r="1119" spans="1:8" s="50" customFormat="1" x14ac:dyDescent="0.2">
@@ -22531,7 +22531,7 @@
       </c>
       <c r="G1122" s="51"/>
       <c r="H1122" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
     </row>
     <row r="1123" spans="1:8" s="50" customFormat="1" x14ac:dyDescent="0.2">
@@ -22899,7 +22899,7 @@
     </row>
     <row r="1141" spans="1:7" s="50" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1141" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="B1141" s="51">
         <v>1.6913846153846155E-10</v>
@@ -25656,7 +25656,7 @@
     </row>
     <row r="1316" spans="1:8" s="50" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1316" s="50" t="s">
-        <v>406</v>
+        <v>512</v>
       </c>
       <c r="B1316" s="50">
         <v>1</v>
@@ -26089,7 +26089,7 @@
     </row>
     <row r="1354" spans="1:12" s="50" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1354" s="50" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="B1354" s="50">
         <f>1/560000</f>
@@ -26099,7 +26099,7 @@
         <v>7</v>
       </c>
       <c r="E1354" s="50" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="F1354" s="50" t="s">
         <v>27</v>
@@ -26508,7 +26508,7 @@
     </row>
     <row r="1378" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1378" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="B1378" s="2">
         <v>2</v>
@@ -26517,7 +26517,7 @@
         <v>17</v>
       </c>
       <c r="E1378" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="F1378" t="s">
         <v>27</v>
@@ -30631,7 +30631,7 @@
     </row>
     <row r="1613" spans="1:15" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A1613" s="53" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="B1613" s="59">
         <f>1/120</f>
@@ -30647,7 +30647,7 @@
         <v>18</v>
       </c>
       <c r="H1613" s="53" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="K1613" s="57"/>
       <c r="L1613"/>
@@ -31137,7 +31137,7 @@
     </row>
     <row r="1640" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1640" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="B1640" s="2">
         <v>2</v>
@@ -31146,7 +31146,7 @@
         <v>17</v>
       </c>
       <c r="E1640" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="F1640" t="s">
         <v>27</v>
@@ -33116,7 +33116,7 @@
         <v>0</v>
       </c>
       <c r="B1754" s="1" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="C1754" s="53"/>
       <c r="D1754" s="53"/>
@@ -33565,7 +33565,7 @@
     </row>
     <row r="1778" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1778" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="B1778" s="3">
         <v>7.1789570411210658E-8</v>
@@ -34023,7 +34023,7 @@
         <v>0</v>
       </c>
       <c r="B1804" s="1" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="C1804" s="53"/>
       <c r="D1804" s="53"/>
@@ -34255,7 +34255,7 @@
     </row>
     <row r="1816" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1816" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="B1816" s="3">
         <v>2.3599288167039204E-6</v>
@@ -34507,7 +34507,7 @@
     </row>
     <row r="1830" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1830" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="B1830" s="3">
         <v>9.7553481893140337E-8</v>
@@ -35017,7 +35017,7 @@
         <v>0</v>
       </c>
       <c r="B1859" s="1" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="C1859" s="53"/>
       <c r="D1859" s="53"/>
@@ -35169,16 +35169,16 @@
         <v>3</v>
       </c>
       <c r="H1867" t="s">
+        <v>479</v>
+      </c>
+      <c r="I1867" t="s">
+        <v>497</v>
+      </c>
+      <c r="J1867" t="s">
         <v>480</v>
       </c>
-      <c r="I1867" t="s">
-        <v>498</v>
-      </c>
-      <c r="J1867" t="s">
+      <c r="K1867" t="s">
         <v>481</v>
-      </c>
-      <c r="K1867" t="s">
-        <v>482</v>
       </c>
     </row>
     <row r="1868" spans="1:12" x14ac:dyDescent="0.2">
@@ -35559,7 +35559,7 @@
         <v>0</v>
       </c>
       <c r="B1885" s="1" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="C1885" s="53"/>
       <c r="D1885" s="53"/>
@@ -35591,7 +35591,7 @@
         <v>9</v>
       </c>
       <c r="B1887" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="C1887" s="53"/>
       <c r="D1887" s="53"/>
@@ -35713,16 +35713,16 @@
         <v>3</v>
       </c>
       <c r="H1893" t="s">
+        <v>479</v>
+      </c>
+      <c r="I1893" t="s">
+        <v>497</v>
+      </c>
+      <c r="J1893" t="s">
         <v>480</v>
       </c>
-      <c r="I1893" t="s">
-        <v>498</v>
-      </c>
-      <c r="J1893" t="s">
+      <c r="K1893" t="s">
         <v>481</v>
-      </c>
-      <c r="K1893" t="s">
-        <v>482</v>
       </c>
     </row>
     <row r="1894" spans="1:12" x14ac:dyDescent="0.2">
@@ -35803,7 +35803,7 @@
         <v>5</v>
       </c>
       <c r="I1896">
-        <f>B1896</f>
+        <f t="shared" ref="I1896:I1901" si="0">B1896</f>
         <v>5.9933333333333334E-4</v>
       </c>
       <c r="J1896">
@@ -35838,7 +35838,7 @@
         <v>5</v>
       </c>
       <c r="I1897">
-        <f>B1897</f>
+        <f t="shared" si="0"/>
         <v>2.9804347826086958E-5</v>
       </c>
       <c r="J1897">
@@ -35874,7 +35874,7 @@
         <v>5</v>
       </c>
       <c r="I1898">
-        <f>B1898</f>
+        <f t="shared" si="0"/>
         <v>5.9599999999999992E-5</v>
       </c>
       <c r="J1898">
@@ -35909,7 +35909,7 @@
         <v>5</v>
       </c>
       <c r="I1899">
-        <f>B1899</f>
+        <f t="shared" si="0"/>
         <v>2.6492753623188407E-5</v>
       </c>
       <c r="J1899">
@@ -35923,7 +35923,7 @@
     </row>
     <row r="1900" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1900" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B1900">
         <f>48/200000/0.75</f>
@@ -35939,13 +35939,13 @@
         <v>18</v>
       </c>
       <c r="G1900" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="H1900">
         <v>5</v>
       </c>
       <c r="I1900">
-        <f>B1900</f>
+        <f t="shared" si="0"/>
         <v>3.2000000000000003E-4</v>
       </c>
       <c r="J1900">
@@ -35981,7 +35981,7 @@
         <v>5</v>
       </c>
       <c r="I1901">
-        <f>B1901</f>
+        <f t="shared" si="0"/>
         <v>3.9733333333333335E-5</v>
       </c>
       <c r="J1901">
@@ -36001,7 +36001,7 @@
         <v>0</v>
       </c>
       <c r="B1903" s="60" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="1904" spans="1:12" x14ac:dyDescent="0.2">
@@ -36042,7 +36042,7 @@
         <v>8</v>
       </c>
       <c r="B1908" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="1909" spans="1:12" x14ac:dyDescent="0.2">
@@ -36050,7 +36050,7 @@
         <v>9</v>
       </c>
       <c r="B1909" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
     </row>
     <row r="1910" spans="1:12" ht="16" x14ac:dyDescent="0.2">
@@ -36114,7 +36114,7 @@
     </row>
     <row r="1913" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1913" s="65" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="B1913" s="66">
         <v>3</v>
@@ -36129,12 +36129,12 @@
         <v>18</v>
       </c>
       <c r="H1913" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="1914" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1914" s="65" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="B1914" s="66">
         <f>15900*(B1913/1000)</f>
@@ -36150,7 +36150,7 @@
         <v>18</v>
       </c>
       <c r="H1914" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1915" spans="1:12" x14ac:dyDescent="0.2">
@@ -36176,7 +36176,7 @@
     </row>
     <row r="1916" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1916" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="B1916" s="66">
         <f>-1*B1913</f>
@@ -36192,7 +36192,7 @@
         <v>18</v>
       </c>
       <c r="H1916" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="1917" spans="1:12" x14ac:dyDescent="0.2">
@@ -36203,7 +36203,7 @@
         <v>0</v>
       </c>
       <c r="B1918" s="1" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="C1918" s="53"/>
       <c r="D1918" s="53"/>
@@ -36357,16 +36357,16 @@
         <v>3</v>
       </c>
       <c r="H1926" t="s">
+        <v>479</v>
+      </c>
+      <c r="I1926" t="s">
+        <v>497</v>
+      </c>
+      <c r="J1926" t="s">
         <v>480</v>
       </c>
-      <c r="I1926" t="s">
-        <v>498</v>
-      </c>
-      <c r="J1926" t="s">
+      <c r="K1926" t="s">
         <v>481</v>
-      </c>
-      <c r="K1926" t="s">
-        <v>482</v>
       </c>
     </row>
     <row r="1927" spans="1:15" x14ac:dyDescent="0.2">
@@ -36399,7 +36399,7 @@
     </row>
     <row r="1928" spans="1:15" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A1928" s="53" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="B1928" s="59">
         <f>1/120</f>
@@ -36415,7 +36415,7 @@
         <v>18</v>
       </c>
       <c r="G1928" s="53" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="K1928" s="57"/>
       <c r="L1928"/>
@@ -36593,7 +36593,7 @@
     </row>
     <row r="1935" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A1935" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B1935" s="28">
         <f>(23.75*0.2)/1.8/200000</f>
@@ -36609,7 +36609,7 @@
         <v>18</v>
       </c>
       <c r="G1935" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="H1935">
         <v>5</v>
@@ -36704,7 +36704,7 @@
         <v>0</v>
       </c>
       <c r="B1939" s="1" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="1940" spans="1:11" x14ac:dyDescent="0.2">
@@ -36712,7 +36712,7 @@
         <v>9</v>
       </c>
       <c r="B1940" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="1941" spans="1:11" x14ac:dyDescent="0.2">
@@ -36720,7 +36720,7 @@
         <v>396</v>
       </c>
       <c r="B1941" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="1942" spans="1:11" x14ac:dyDescent="0.2">
@@ -36794,7 +36794,7 @@
     </row>
     <row r="1949" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1949" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="B1949">
         <v>1</v>
@@ -36814,7 +36814,7 @@
     </row>
     <row r="1950" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1950" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="B1950">
         <v>8.4039805756723712E-6</v>
@@ -36829,12 +36829,12 @@
         <v>18</v>
       </c>
       <c r="G1950" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="1951" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1951" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="B1951">
         <v>1.3427927506200167E-4</v>
@@ -36849,7 +36849,7 @@
         <v>18</v>
       </c>
       <c r="G1951" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="1952" spans="1:11" x14ac:dyDescent="0.2">
@@ -37110,7 +37110,7 @@
     </row>
     <row r="1966" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1966" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="B1966" s="3">
         <v>7.1789570411210658E-8</v>
@@ -37563,7 +37563,7 @@
         <v>0</v>
       </c>
       <c r="B1993" s="1" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="1994" spans="1:8" x14ac:dyDescent="0.2">
@@ -37571,7 +37571,7 @@
         <v>9</v>
       </c>
       <c r="B1994" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="1995" spans="1:8" x14ac:dyDescent="0.2">
@@ -37579,7 +37579,7 @@
         <v>396</v>
       </c>
       <c r="B1995" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="1996" spans="1:8" x14ac:dyDescent="0.2">
@@ -37611,7 +37611,7 @@
         <v>8</v>
       </c>
       <c r="B1999" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="2000" spans="1:8" x14ac:dyDescent="0.2">
@@ -37659,21 +37659,21 @@
         <v>3</v>
       </c>
       <c r="H2003" t="s">
+        <v>479</v>
+      </c>
+      <c r="I2003" t="s">
+        <v>497</v>
+      </c>
+      <c r="J2003" t="s">
         <v>480</v>
       </c>
-      <c r="I2003" t="s">
-        <v>498</v>
-      </c>
-      <c r="J2003" t="s">
+      <c r="K2003" t="s">
         <v>481</v>
-      </c>
-      <c r="K2003" t="s">
-        <v>482</v>
       </c>
     </row>
     <row r="2004" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2004" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="B2004">
         <v>1</v>
@@ -37756,7 +37756,7 @@
     </row>
     <row r="2007" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2007" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="B2007">
         <v>1.2763976504487801E-4</v>
@@ -37771,7 +37771,7 @@
         <v>18</v>
       </c>
       <c r="G2007" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="H2007">
         <v>5</v>
@@ -38034,7 +38034,7 @@
         <v>0</v>
       </c>
       <c r="B2022" s="1" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="2023" spans="1:10" x14ac:dyDescent="0.2">
@@ -38042,7 +38042,7 @@
         <v>9</v>
       </c>
       <c r="B2023" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="2024" spans="1:10" x14ac:dyDescent="0.2">
@@ -38050,7 +38050,7 @@
         <v>396</v>
       </c>
       <c r="B2024" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="2025" spans="1:10" x14ac:dyDescent="0.2">
@@ -38082,7 +38082,7 @@
         <v>8</v>
       </c>
       <c r="B2028" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="2029" spans="1:10" x14ac:dyDescent="0.2">
@@ -38127,21 +38127,21 @@
         <v>3</v>
       </c>
       <c r="G2032" t="s">
+        <v>479</v>
+      </c>
+      <c r="H2032" t="s">
+        <v>497</v>
+      </c>
+      <c r="I2032" t="s">
         <v>480</v>
       </c>
-      <c r="H2032" t="s">
-        <v>498</v>
-      </c>
-      <c r="I2032" t="s">
+      <c r="J2032" t="s">
         <v>481</v>
-      </c>
-      <c r="J2032" t="s">
-        <v>482</v>
       </c>
     </row>
     <row r="2033" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2033" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="B2033">
         <v>1</v>
@@ -38209,7 +38209,7 @@
         <v>5</v>
       </c>
       <c r="H2035">
-        <f>B2035</f>
+        <f t="shared" ref="H2035:H2040" si="1">B2035</f>
         <v>5.8548009367681507E-6</v>
       </c>
       <c r="I2035">
@@ -38244,7 +38244,7 @@
         <v>5</v>
       </c>
       <c r="H2036">
-        <f>B2036</f>
+        <f t="shared" si="1"/>
         <v>2.0319944081098179E-5</v>
       </c>
       <c r="I2036">
@@ -38279,7 +38279,7 @@
         <v>5</v>
       </c>
       <c r="H2037">
-        <f>B2037</f>
+        <f t="shared" si="1"/>
         <v>2.9685693565181665E-6</v>
       </c>
       <c r="I2037">
@@ -38314,7 +38314,7 @@
         <v>5</v>
       </c>
       <c r="H2038">
-        <f>B2038</f>
+        <f t="shared" si="1"/>
         <v>8.4309133489461356E-6</v>
       </c>
       <c r="I2038">
@@ -38328,7 +38328,7 @@
     </row>
     <row r="2039" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2039" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B2039">
         <f>399/700000/6.1</f>
@@ -38344,13 +38344,13 @@
         <v>18</v>
       </c>
       <c r="F2039" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="G2039">
         <v>5</v>
       </c>
       <c r="H2039">
-        <f>B2039</f>
+        <f t="shared" si="1"/>
         <v>9.3442622950819676E-5</v>
       </c>
       <c r="I2039">
@@ -38364,7 +38364,7 @@
     </row>
     <row r="2040" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2040" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="B2040">
         <f>4.16666666666667E-08*10/6.1</f>
@@ -38380,13 +38380,13 @@
         <v>18</v>
       </c>
       <c r="F2040" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="G2040">
         <v>5</v>
       </c>
       <c r="H2040">
-        <f>B2040</f>
+        <f t="shared" si="1"/>
         <v>6.8306010928961812E-8</v>
       </c>
       <c r="I2040">
@@ -38403,7 +38403,7 @@
         <v>0</v>
       </c>
       <c r="B2042" s="1" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="2043" spans="1:10" x14ac:dyDescent="0.2">
@@ -38419,7 +38419,7 @@
         <v>396</v>
       </c>
       <c r="B2044" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="2045" spans="1:10" x14ac:dyDescent="0.2">
@@ -38443,7 +38443,7 @@
         <v>3</v>
       </c>
       <c r="B2047" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="2048" spans="1:10" x14ac:dyDescent="0.2">
@@ -38451,7 +38451,7 @@
         <v>8</v>
       </c>
       <c r="B2048" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
     </row>
     <row r="2049" spans="1:8" x14ac:dyDescent="0.2">
@@ -38507,18 +38507,18 @@
         <v>3</v>
       </c>
       <c r="H2053" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="2054" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2054" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="B2054">
         <v>1</v>
       </c>
       <c r="C2054" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="D2054" t="s">
         <v>103</v>
@@ -38530,21 +38530,21 @@
         <v>15</v>
       </c>
       <c r="G2054" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="H2054" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="2055" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2055" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="B2055">
         <v>4.3</v>
       </c>
       <c r="C2055" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="D2055" t="s">
         <v>103</v>
@@ -38556,21 +38556,21 @@
         <v>18</v>
       </c>
       <c r="G2055" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="H2055" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="2056" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2056" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="B2056">
         <v>1</v>
       </c>
       <c r="C2056" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="D2056" t="s">
         <v>103</v>
@@ -38582,21 +38582,21 @@
         <v>18</v>
       </c>
       <c r="G2056" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="H2056" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="2057" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2057" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="B2057">
         <v>1</v>
       </c>
       <c r="C2057" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="D2057" t="s">
         <v>103</v>
@@ -38608,10 +38608,10 @@
         <v>18</v>
       </c>
       <c r="G2057" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="H2057" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="2058" spans="1:8" x14ac:dyDescent="0.2">
@@ -38622,7 +38622,7 @@
         <v>0</v>
       </c>
       <c r="B2059" s="1" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="2060" spans="1:8" x14ac:dyDescent="0.2">
@@ -38630,7 +38630,7 @@
         <v>9</v>
       </c>
       <c r="B2060" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="2061" spans="1:8" x14ac:dyDescent="0.2">
@@ -38638,7 +38638,7 @@
         <v>396</v>
       </c>
       <c r="B2061" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="2062" spans="1:8" x14ac:dyDescent="0.2">
@@ -38670,7 +38670,7 @@
         <v>8</v>
       </c>
       <c r="B2065" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="2066" spans="1:10" x14ac:dyDescent="0.2">
@@ -38715,21 +38715,21 @@
         <v>3</v>
       </c>
       <c r="G2069" t="s">
+        <v>479</v>
+      </c>
+      <c r="H2069" t="s">
+        <v>497</v>
+      </c>
+      <c r="I2069" t="s">
         <v>480</v>
       </c>
-      <c r="H2069" t="s">
-        <v>498</v>
-      </c>
-      <c r="I2069" t="s">
+      <c r="J2069" t="s">
         <v>481</v>
-      </c>
-      <c r="J2069" t="s">
-        <v>482</v>
       </c>
     </row>
     <row r="2070" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2070" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="B2070">
         <v>1</v>
@@ -38752,7 +38752,7 @@
     </row>
     <row r="2071" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A2071" s="53" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="B2071" s="59">
         <f>1/120</f>
@@ -38768,7 +38768,7 @@
         <v>18</v>
       </c>
       <c r="F2071" s="53" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="G2071" s="53">
         <v>0</v>
@@ -38869,7 +38869,7 @@
         <v>5</v>
       </c>
       <c r="H2074">
-        <f t="shared" ref="H2074" si="0">B2074</f>
+        <f t="shared" ref="H2074" si="2">B2074</f>
         <v>5.6689342403628128E-6</v>
       </c>
       <c r="I2074">
@@ -38904,7 +38904,7 @@
         <v>5</v>
       </c>
       <c r="H2075">
-        <f t="shared" ref="H2075" si="1">B2075</f>
+        <f t="shared" ref="H2075" si="3">B2075</f>
         <v>2.4040391954934648E-5</v>
       </c>
       <c r="I2075">
@@ -38939,7 +38939,7 @@
         <v>5</v>
       </c>
       <c r="H2076">
-        <f t="shared" ref="H2076" si="2">B2076</f>
+        <f t="shared" ref="H2076" si="4">B2076</f>
         <v>3.1830926606374987E-6</v>
       </c>
       <c r="I2076">
@@ -38974,7 +38974,7 @@
         <v>5</v>
       </c>
       <c r="H2077">
-        <f t="shared" ref="H2077" si="3">B2077</f>
+        <f t="shared" ref="H2077" si="5">B2077</f>
         <v>8.16326530612245E-6</v>
       </c>
       <c r="I2077">
@@ -38988,7 +38988,7 @@
     </row>
     <row r="2078" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2078" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B2078">
         <f>80/700000/6.3</f>
@@ -39004,7 +39004,7 @@
         <v>18</v>
       </c>
       <c r="F2078" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="G2078">
         <v>5</v>
@@ -39030,7 +39030,7 @@
         <v>0</v>
       </c>
       <c r="B2080" s="1" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="2081" spans="1:10" x14ac:dyDescent="0.2">
@@ -39038,7 +39038,7 @@
         <v>9</v>
       </c>
       <c r="B2081" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="2082" spans="1:10" x14ac:dyDescent="0.2">
@@ -39046,7 +39046,7 @@
         <v>396</v>
       </c>
       <c r="B2082" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="2083" spans="1:10" x14ac:dyDescent="0.2">
@@ -39078,7 +39078,7 @@
         <v>8</v>
       </c>
       <c r="B2086" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="2087" spans="1:10" x14ac:dyDescent="0.2">
@@ -39123,21 +39123,21 @@
         <v>3</v>
       </c>
       <c r="G2090" s="60" t="s">
+        <v>479</v>
+      </c>
+      <c r="H2090" s="60" t="s">
+        <v>497</v>
+      </c>
+      <c r="I2090" s="60" t="s">
         <v>480</v>
       </c>
-      <c r="H2090" s="60" t="s">
-        <v>498</v>
-      </c>
-      <c r="I2090" s="60" t="s">
+      <c r="J2090" s="60" t="s">
         <v>481</v>
-      </c>
-      <c r="J2090" s="60" t="s">
-        <v>482</v>
       </c>
     </row>
     <row r="2091" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2091" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="B2091">
         <v>1</v>
@@ -39205,15 +39205,15 @@
         <v>5</v>
       </c>
       <c r="H2093">
-        <f t="shared" ref="H2093:H2095" si="4">B2093</f>
+        <f t="shared" ref="H2093:H2095" si="6">B2093</f>
         <v>4.3859649122807014E-6</v>
       </c>
       <c r="I2093">
-        <f t="shared" ref="I2093:I2095" si="5">B2093*(1000000/1250000)</f>
+        <f t="shared" ref="I2093:I2095" si="7">B2093*(1000000/1250000)</f>
         <v>3.5087719298245615E-6</v>
       </c>
       <c r="J2093">
-        <f t="shared" ref="J2093:J2095" si="6">B2093*(1000000/750000)</f>
+        <f t="shared" ref="J2093:J2095" si="8">B2093*(1000000/750000)</f>
         <v>5.8479532163742686E-6</v>
       </c>
     </row>
@@ -39240,15 +39240,15 @@
         <v>5</v>
       </c>
       <c r="H2094">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>1.529271460518488E-5</v>
       </c>
       <c r="I2094">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1.2234171684147905E-5</v>
       </c>
       <c r="J2094">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>2.0390286140246506E-5</v>
       </c>
     </row>
@@ -39275,15 +39275,15 @@
         <v>5</v>
       </c>
       <c r="H2095">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2.2293376104859981E-6</v>
       </c>
       <c r="I2095">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1.7834700883887986E-6</v>
       </c>
       <c r="J2095">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>2.9724501473146639E-6</v>
       </c>
     </row>
@@ -39324,7 +39324,7 @@
     </row>
     <row r="2097" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2097" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="B2097">
         <f>66/1000000/5.7</f>
@@ -39340,7 +39340,7 @@
         <v>18</v>
       </c>
       <c r="F2097" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="G2097">
         <v>5</v>
@@ -39363,7 +39363,7 @@
         <v>0</v>
       </c>
       <c r="B2099" s="1" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="2100" spans="1:10" x14ac:dyDescent="0.2">
@@ -39426,7 +39426,7 @@
     </row>
     <row r="2106" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2106" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="B2106">
         <v>1</v>
@@ -39446,7 +39446,7 @@
     </row>
     <row r="2107" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2107" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="B2107" s="2">
         <f>1/(0.089775*3.6)</f>
@@ -39456,13 +39456,13 @@
         <v>104</v>
       </c>
       <c r="D2107" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="E2107" t="s">
         <v>18</v>
       </c>
       <c r="F2107" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="2108" spans="1:10" x14ac:dyDescent="0.2">
@@ -39473,7 +39473,7 @@
         <v>0</v>
       </c>
       <c r="B2109" s="60" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="2110" spans="1:10" x14ac:dyDescent="0.2">
@@ -39513,7 +39513,7 @@
         <v>8</v>
       </c>
       <c r="B2114" s="3" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="2115" spans="1:12" x14ac:dyDescent="0.2">
@@ -39521,7 +39521,7 @@
         <v>9</v>
       </c>
       <c r="B2115" s="3" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="2116" spans="1:12" x14ac:dyDescent="0.2">
@@ -39555,21 +39555,21 @@
         <v>3</v>
       </c>
       <c r="I2117" s="60" t="s">
+        <v>479</v>
+      </c>
+      <c r="J2117" s="60" t="s">
+        <v>497</v>
+      </c>
+      <c r="K2117" s="60" t="s">
         <v>480</v>
       </c>
-      <c r="J2117" s="60" t="s">
-        <v>498</v>
-      </c>
-      <c r="K2117" s="60" t="s">
+      <c r="L2117" s="60" t="s">
         <v>481</v>
-      </c>
-      <c r="L2117" s="60" t="s">
-        <v>482</v>
       </c>
     </row>
     <row r="2118" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2118" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="B2118" s="3">
         <v>1</v>
@@ -39619,7 +39619,7 @@
     </row>
     <row r="2120" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2120" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="B2120" s="3">
         <v>9.5816828884557961E-5</v>
@@ -39634,10 +39634,10 @@
         <v>18</v>
       </c>
       <c r="G2120" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="H2120" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="I2120">
         <v>0</v>
@@ -39645,7 +39645,7 @@
     </row>
     <row r="2121" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2121" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B2121">
         <f>8.1/38500/(0.0753*3.6)</f>
@@ -39661,7 +39661,7 @@
         <v>18</v>
       </c>
       <c r="H2121" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="I2121">
         <v>5</v>
@@ -39684,7 +39684,7 @@
         <v>0</v>
       </c>
       <c r="B2123" s="60" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="2124" spans="1:12" x14ac:dyDescent="0.2">
@@ -39724,7 +39724,7 @@
         <v>8</v>
       </c>
       <c r="B2128" s="3" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="2129" spans="1:15" x14ac:dyDescent="0.2">
@@ -39732,7 +39732,7 @@
         <v>9</v>
       </c>
       <c r="B2129" s="3" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="2130" spans="1:15" x14ac:dyDescent="0.2">
@@ -39766,21 +39766,21 @@
         <v>3</v>
       </c>
       <c r="I2131" s="60" t="s">
+        <v>479</v>
+      </c>
+      <c r="J2131" s="60" t="s">
+        <v>497</v>
+      </c>
+      <c r="K2131" s="60" t="s">
         <v>480</v>
       </c>
-      <c r="J2131" s="60" t="s">
-        <v>498</v>
-      </c>
-      <c r="K2131" s="60" t="s">
+      <c r="L2131" s="60" t="s">
         <v>481</v>
-      </c>
-      <c r="L2131" s="60" t="s">
-        <v>482</v>
       </c>
     </row>
     <row r="2132" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A2132" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="B2132" s="3">
         <v>1</v>
@@ -39822,7 +39822,7 @@
         <v>18</v>
       </c>
       <c r="G2133" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="H2133" s="55" t="s">
         <v>389</v>
@@ -39862,7 +39862,7 @@
         <v>18</v>
       </c>
       <c r="G2134" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="H2134" t="s">
         <v>399</v>
@@ -39885,7 +39885,7 @@
     </row>
     <row r="2135" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A2135" s="53" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="B2135" s="62">
         <f>1/120</f>
@@ -39901,7 +39901,7 @@
         <v>18</v>
       </c>
       <c r="H2135" s="53" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="I2135">
         <v>0</v>
@@ -39909,7 +39909,7 @@
     </row>
     <row r="2136" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A2136" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B2136">
         <f>(8.1/5)/38500/(0.0753*3.6)</f>
@@ -39925,7 +39925,7 @@
         <v>18</v>
       </c>
       <c r="H2136" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="I2136">
         <v>5</v>
@@ -39948,7 +39948,7 @@
         <v>0</v>
       </c>
       <c r="B2138" s="1" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="C2138" s="53"/>
       <c r="D2138" s="53"/>
@@ -40160,7 +40160,7 @@
     </row>
     <row r="2149" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2149" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="B2149" s="3">
         <v>8.8450704225352119E-4</v>
@@ -40304,7 +40304,7 @@
     </row>
     <row r="2157" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2157" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="B2157" s="3">
         <v>1.4133139635978708E-6</v>
@@ -40322,7 +40322,7 @@
     </row>
     <row r="2158" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2158" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="B2158" s="3">
         <v>6.1476482081469075E-6</v>
@@ -40430,7 +40430,7 @@
     </row>
     <row r="2164" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2164" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="B2164" s="3">
         <v>1.5491421214163292E-7</v>
@@ -40466,7 +40466,7 @@
     </row>
     <row r="2166" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2166" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="B2166" s="3">
         <v>9.9199451634554413E-7</v>
@@ -40718,7 +40718,7 @@
     </row>
     <row r="2180" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2180" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="B2180" s="3">
         <v>7.0588235294117658E-12</v>
@@ -40736,7 +40736,7 @@
     </row>
     <row r="2181" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2181" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="B2181" s="3">
         <v>4.7058823529411767E-12</v>
@@ -40754,7 +40754,7 @@
     </row>
     <row r="2182" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2182" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="B2182" s="3">
         <v>5.082352941176471E-8</v>
@@ -40772,7 +40772,7 @@
     </row>
     <row r="2183" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2183" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B2183" s="3">
         <v>9.8823529411764698E-10</v>
@@ -40790,7 +40790,7 @@
     </row>
     <row r="2184" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2184" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B2184" s="3">
         <v>3.0588235294117649E-10</v>
@@ -40808,7 +40808,7 @@
     </row>
     <row r="2185" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2185" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="B2185" s="3">
         <v>3.7647058823529416E-10</v>
@@ -40844,7 +40844,7 @@
     </row>
     <row r="2187" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2187" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="B2187" s="3">
         <v>2.0470588235294119E-10</v>
@@ -40862,7 +40862,7 @@
     </row>
     <row r="2188" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2188" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="B2188" s="3">
         <v>2.5411764705882359E-10</v>
@@ -40883,7 +40883,7 @@
         <v>0</v>
       </c>
       <c r="B2190" s="1" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="2191" spans="1:8" x14ac:dyDescent="0.2">
@@ -40931,7 +40931,7 @@
         <v>8</v>
       </c>
       <c r="B2196" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="2197" spans="1:11" x14ac:dyDescent="0.2">
@@ -40939,7 +40939,7 @@
         <v>396</v>
       </c>
       <c r="B2197" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="2198" spans="1:11" x14ac:dyDescent="0.2">
@@ -40947,7 +40947,7 @@
         <v>9</v>
       </c>
       <c r="B2198" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="2199" spans="1:11" ht="16" x14ac:dyDescent="0.2">
@@ -40979,21 +40979,21 @@
         <v>3</v>
       </c>
       <c r="H2200" s="60" t="s">
+        <v>479</v>
+      </c>
+      <c r="I2200" s="60" t="s">
+        <v>497</v>
+      </c>
+      <c r="J2200" s="60" t="s">
         <v>480</v>
       </c>
-      <c r="I2200" s="60" t="s">
-        <v>498</v>
-      </c>
-      <c r="J2200" s="60" t="s">
+      <c r="K2200" s="60" t="s">
         <v>481</v>
-      </c>
-      <c r="K2200" s="60" t="s">
-        <v>482</v>
       </c>
     </row>
     <row r="2201" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A2201" s="64" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="B2201">
         <v>1</v>
@@ -41016,7 +41016,7 @@
     </row>
     <row r="2202" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2202" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="B2202">
         <v>1.1278940455009136E-4</v>
@@ -41034,7 +41034,7 @@
         <v>18</v>
       </c>
       <c r="G2202" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="H2202">
         <v>5</v>
@@ -41054,7 +41054,7 @@
     </row>
     <row r="2203" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2203" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="B2203">
         <v>3.8539996192328446E-6</v>
@@ -41072,7 +41072,7 @@
         <v>18</v>
       </c>
       <c r="G2203" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="2204" spans="1:11" x14ac:dyDescent="0.2">
@@ -41115,7 +41115,7 @@
     </row>
     <row r="2206" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2206" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="B2206">
         <v>8.8352086295850824E-8</v>
@@ -41268,7 +41268,7 @@
     </row>
     <row r="2215" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2215" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="B2215">
         <v>2.6338739709305827E-6</v>
@@ -41302,7 +41302,7 @@
     </row>
     <row r="2217" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2217" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="B2217">
         <v>1.229967209887436E-10</v>
@@ -41319,7 +41319,7 @@
     </row>
     <row r="2218" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2218" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B2218">
         <v>2.0499453498123931E-10</v>
@@ -41336,7 +41336,7 @@
     </row>
     <row r="2219" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2219" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="B2219">
         <v>1.9486966093412831E-6</v>
@@ -41370,7 +41370,7 @@
     </row>
     <row r="2221" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2221" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="B2221">
         <v>2.3299378853965246E-12</v>
@@ -41404,7 +41404,7 @@
     </row>
     <row r="2223" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2223" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="B2223">
         <v>2.0199461495712361E-10</v>
@@ -41455,7 +41455,7 @@
     </row>
     <row r="2226" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2226" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="B2226">
         <v>3.3193620217056908E-6</v>
@@ -41489,7 +41489,7 @@
     </row>
     <row r="2228" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2228" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="B2228">
         <v>2.3299378853965246E-12</v>
@@ -41574,7 +41574,7 @@
     </row>
     <row r="2233" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2233" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="B2233">
         <v>4.0498920325561916E-8</v>
@@ -41625,7 +41625,7 @@
     </row>
     <row r="2236" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2236" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="B2236">
         <v>6.9798139227758525E-10</v>
@@ -41659,7 +41659,7 @@
     </row>
     <row r="2238" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2238" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B2238">
         <v>4.9298685729634615E-10</v>
@@ -41696,7 +41696,7 @@
         <v>0</v>
       </c>
       <c r="B2242" s="1" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="2243" spans="1:11" x14ac:dyDescent="0.2">
@@ -41744,7 +41744,7 @@
         <v>8</v>
       </c>
       <c r="B2248" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="2249" spans="1:11" x14ac:dyDescent="0.2">
@@ -41752,7 +41752,7 @@
         <v>396</v>
       </c>
       <c r="B2249" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="2250" spans="1:11" x14ac:dyDescent="0.2">
@@ -41760,7 +41760,7 @@
         <v>9</v>
       </c>
       <c r="B2250" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
     </row>
     <row r="2251" spans="1:11" ht="16" x14ac:dyDescent="0.2">
@@ -41792,21 +41792,21 @@
         <v>3</v>
       </c>
       <c r="H2252" t="s">
+        <v>479</v>
+      </c>
+      <c r="I2252" t="s">
+        <v>497</v>
+      </c>
+      <c r="J2252" t="s">
         <v>480</v>
       </c>
-      <c r="I2252" t="s">
-        <v>498</v>
-      </c>
-      <c r="J2252" t="s">
+      <c r="K2252" t="s">
         <v>481</v>
-      </c>
-      <c r="K2252" t="s">
-        <v>482</v>
       </c>
     </row>
     <row r="2253" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A2253" s="64" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="B2253">
         <v>1</v>
@@ -41984,7 +41984,7 @@
     </row>
     <row r="2258" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2258" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B2258">
         <f>283/710000/5.45</f>
@@ -42000,7 +42000,7 @@
         <v>18</v>
       </c>
       <c r="G2258" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="H2258">
         <v>5</v>
@@ -42026,7 +42026,7 @@
         <v>0</v>
       </c>
       <c r="B2260" s="1" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="2261" spans="1:11" x14ac:dyDescent="0.2">
@@ -42074,7 +42074,7 @@
         <v>8</v>
       </c>
       <c r="B2266" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="2267" spans="1:11" x14ac:dyDescent="0.2">
@@ -42082,7 +42082,7 @@
         <v>396</v>
       </c>
       <c r="B2267" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="2268" spans="1:11" x14ac:dyDescent="0.2">
@@ -42090,7 +42090,7 @@
         <v>9</v>
       </c>
       <c r="B2268" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
     </row>
     <row r="2269" spans="1:11" ht="16" x14ac:dyDescent="0.2">
@@ -42122,21 +42122,21 @@
         <v>3</v>
       </c>
       <c r="H2270" t="s">
+        <v>479</v>
+      </c>
+      <c r="I2270" t="s">
+        <v>497</v>
+      </c>
+      <c r="J2270" t="s">
         <v>480</v>
       </c>
-      <c r="I2270" t="s">
-        <v>498</v>
-      </c>
-      <c r="J2270" t="s">
+      <c r="K2270" t="s">
         <v>481</v>
-      </c>
-      <c r="K2270" t="s">
-        <v>482</v>
       </c>
     </row>
     <row r="2271" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A2271" s="64" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="B2271">
         <v>1</v>
@@ -42162,7 +42162,7 @@
     </row>
     <row r="2272" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A2272" s="53" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="B2272" s="62">
         <f>1/120</f>
@@ -42178,7 +42178,7 @@
         <v>18</v>
       </c>
       <c r="G2272" s="53" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="H2272">
         <v>0</v>
@@ -42384,7 +42384,7 @@
         <v>5</v>
       </c>
       <c r="I2278">
-        <f t="shared" ref="I2278:I2279" si="7">B2278</f>
+        <f t="shared" ref="I2278:I2279" si="9">B2278</f>
         <v>1.178082191780822E-5</v>
       </c>
       <c r="J2278">
@@ -42398,7 +42398,7 @@
     </row>
     <row r="2279" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2279" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B2279">
         <f>47/1000000/11</f>
@@ -42414,13 +42414,13 @@
         <v>18</v>
       </c>
       <c r="G2279" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="H2279">
         <v>5</v>
       </c>
       <c r="I2279">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>4.2727272727272722E-6</v>
       </c>
       <c r="J2279">
@@ -42440,7 +42440,7 @@
         <v>0</v>
       </c>
       <c r="B2282" s="1" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
     </row>
     <row r="2283" spans="1:11" x14ac:dyDescent="0.2">
@@ -42448,7 +42448,7 @@
         <v>9</v>
       </c>
       <c r="B2283" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
     </row>
     <row r="2284" spans="1:11" x14ac:dyDescent="0.2">
@@ -42456,7 +42456,7 @@
         <v>396</v>
       </c>
       <c r="B2284" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="2285" spans="1:11" x14ac:dyDescent="0.2">
@@ -42488,7 +42488,7 @@
         <v>8</v>
       </c>
       <c r="B2288" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="2289" spans="1:11" x14ac:dyDescent="0.2">
@@ -42536,21 +42536,21 @@
         <v>3</v>
       </c>
       <c r="H2292" t="s">
+        <v>479</v>
+      </c>
+      <c r="I2292" t="s">
+        <v>497</v>
+      </c>
+      <c r="J2292" t="s">
         <v>480</v>
       </c>
-      <c r="I2292" t="s">
-        <v>498</v>
-      </c>
-      <c r="J2292" t="s">
+      <c r="K2292" t="s">
         <v>481</v>
-      </c>
-      <c r="K2292" t="s">
-        <v>482</v>
       </c>
     </row>
     <row r="2293" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A2293" s="64" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="B2293">
         <v>1</v>
@@ -42597,7 +42597,7 @@
     </row>
     <row r="2295" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2295" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="B2295">
         <v>1.1510877524470435E-4</v>
@@ -42612,7 +42612,7 @@
         <v>18</v>
       </c>
       <c r="G2295" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="H2295">
         <v>5</v>
@@ -42688,7 +42688,7 @@
     </row>
     <row r="2298" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2298" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="B2298">
         <v>7.891795688303974E-8</v>
@@ -42868,7 +42868,7 @@
     </row>
     <row r="2307" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2307" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="B2307">
         <v>7.63619826432997E-7</v>
@@ -42908,7 +42908,7 @@
     </row>
     <row r="2309" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2309" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="B2309">
         <v>3.9657281817228329E-7</v>
@@ -42988,7 +42988,7 @@
     </row>
     <row r="2313" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2313" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="B2313">
         <v>1.1740772587352886E-5</v>
@@ -43151,7 +43151,7 @@
         <v>0</v>
       </c>
       <c r="B2322" s="1" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
     </row>
     <row r="2323" spans="1:11" x14ac:dyDescent="0.2">
@@ -43159,7 +43159,7 @@
         <v>9</v>
       </c>
       <c r="B2323" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
     </row>
     <row r="2324" spans="1:11" x14ac:dyDescent="0.2">
@@ -43231,16 +43231,16 @@
         <v>3</v>
       </c>
       <c r="H2330" t="s">
+        <v>479</v>
+      </c>
+      <c r="I2330" t="s">
+        <v>497</v>
+      </c>
+      <c r="J2330" t="s">
         <v>480</v>
       </c>
-      <c r="I2330" t="s">
-        <v>498</v>
-      </c>
-      <c r="J2330" t="s">
+      <c r="K2330" t="s">
         <v>481</v>
-      </c>
-      <c r="K2330" t="s">
-        <v>482</v>
       </c>
     </row>
     <row r="2331" spans="1:11" ht="16" x14ac:dyDescent="0.2">
@@ -43271,7 +43271,7 @@
     </row>
     <row r="2332" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2332" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="B2332" s="3">
         <v>1</v>
@@ -43297,7 +43297,7 @@
         <v>0</v>
       </c>
       <c r="B2334" s="1" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
     </row>
     <row r="2335" spans="1:11" x14ac:dyDescent="0.2">
@@ -43305,7 +43305,7 @@
         <v>9</v>
       </c>
       <c r="B2335" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
     </row>
     <row r="2336" spans="1:11" x14ac:dyDescent="0.2">
@@ -43377,16 +43377,16 @@
         <v>3</v>
       </c>
       <c r="H2342" t="s">
+        <v>479</v>
+      </c>
+      <c r="I2342" t="s">
+        <v>497</v>
+      </c>
+      <c r="J2342" t="s">
         <v>480</v>
       </c>
-      <c r="I2342" t="s">
-        <v>498</v>
-      </c>
-      <c r="J2342" t="s">
+      <c r="K2342" t="s">
         <v>481</v>
-      </c>
-      <c r="K2342" t="s">
-        <v>482</v>
       </c>
     </row>
     <row r="2343" spans="1:11" ht="16" x14ac:dyDescent="0.2">
@@ -43417,7 +43417,7 @@
     </row>
     <row r="2344" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2344" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="B2344" s="3">
         <v>1</v>
@@ -43443,7 +43443,7 @@
         <v>0</v>
       </c>
       <c r="B2346" s="1" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
     </row>
     <row r="2347" spans="1:11" x14ac:dyDescent="0.2">
@@ -43451,7 +43451,7 @@
         <v>9</v>
       </c>
       <c r="B2347" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="2348" spans="1:11" x14ac:dyDescent="0.2">
@@ -43523,16 +43523,16 @@
         <v>3</v>
       </c>
       <c r="H2354" t="s">
+        <v>479</v>
+      </c>
+      <c r="I2354" t="s">
+        <v>497</v>
+      </c>
+      <c r="J2354" t="s">
         <v>480</v>
       </c>
-      <c r="I2354" t="s">
-        <v>498</v>
-      </c>
-      <c r="J2354" t="s">
+      <c r="K2354" t="s">
         <v>481</v>
-      </c>
-      <c r="K2354" t="s">
-        <v>482</v>
       </c>
     </row>
     <row r="2355" spans="1:11" ht="16" x14ac:dyDescent="0.2">
@@ -43563,7 +43563,7 @@
     </row>
     <row r="2356" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2356" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="B2356" s="3">
         <v>1</v>
@@ -43578,7 +43578,7 @@
         <v>18</v>
       </c>
       <c r="G2356" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="H2356">
         <v>0</v>

</xml_diff>